<commit_message>
fix: clean drawings/images from excel template to resolve exceljs anchors crash
</commit_message>
<xml_diff>
--- a/.agents/skills/antigravity-prinktech-quote/resources/template_bao_gia.xlsx
+++ b/.agents/skills/antigravity-prinktech-quote/resources/template_bao_gia.xlsx
@@ -625,45 +625,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>1</rowOff>
-    </from>
-    <ext cx="3790950" cy="714374"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="0" y="1"/>
-          <a:ext cx="3790950" cy="714374"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1336,6 +1297,5 @@
     <mergeCell ref="C20:H20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>